<commit_message>
Modelo da planilha de equipe: Nome, CPF, Telefone, Cargo, Cidade, PIX e um dia por coluna
Juan, 09/10/2026 (2ª volta): "CPF, telefone, cargo, cidade, chave Pix e os
dias trabalhados — 10 dias no evento, 10 colunas, com a data e um X ou sim".
O modelo do setor passa a ter Nome, CPF, Telefone, Cargo, Cidade, Chave PIX
e uma coluna para CADA dia do evento (antes só de hoje em diante); X ou SIM
= trabalha, vazio = não, tudo marcado = todos os dias.

O arquivo fixo public/modelo-importacao.xlsx (que aba aberta antes do
deploy ainda baixava, com Valor e uma linha de exemplo com CPF válido que
seria importada) vira a versão genérica do formato novo, sem exemplo.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/modelo-importacao.xlsx
+++ b/public/modelo-importacao.xlsx
@@ -4,6 +4,7 @@
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
     <sheet name="Equipe" sheetId="1" r:id="rId1"/>
+    <sheet name="Como preencher" sheetId="2" r:id="rId2"/>
   </sheets>
 </workbook>
 </file>
@@ -397,15 +398,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:G1"/>
   <cols>
-    <col min="1" max="1" width="30.83203125" customWidth="1"/>
+    <col min="1" max="1" width="34.83203125" customWidth="1"/>
     <col min="2" max="2" width="16.83203125" customWidth="1"/>
     <col min="3" max="3" width="18.83203125" customWidth="1"/>
-    <col min="4" max="4" width="16.83203125" customWidth="1"/>
-    <col min="5" max="5" width="14.83203125" customWidth="1"/>
-    <col min="6" max="6" width="22.83203125" customWidth="1"/>
-    <col min="7" max="7" width="10.83203125" customWidth="1"/>
+    <col min="4" max="4" width="20.83203125" customWidth="1"/>
+    <col min="5" max="5" width="20.83203125" customWidth="1"/>
+    <col min="6" max="6" width="26.83203125" customWidth="1"/>
+    <col min="7" max="7" width="40.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -425,38 +426,79 @@
         <v>Cidade</v>
       </c>
       <c r="F1" t="str">
-        <v>Chave Pix</v>
+        <v>Chave PIX</v>
       </c>
       <c r="G1" t="str">
-        <v>Valor</v>
+        <v>Dias de trabalho</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:G1"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:A10"/>
+  <cols>
+    <col min="1" max="1" width="110.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Como preencher</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>APAGUE ESTA LINHA — exemplo</v>
-      </c>
-      <c r="B2" t="str">
-        <v>123.456.789-09</v>
-      </c>
-      <c r="C2" t="str">
-        <v>(27) 99999-9999</v>
-      </c>
-      <c r="D2" t="str">
-        <v>Barman</v>
-      </c>
-      <c r="E2" t="str">
-        <v>Vitória</v>
-      </c>
-      <c r="F2" t="str">
-        <v>chave@email.com</v>
-      </c>
-      <c r="G2" t="str">
-        <v>150,00</v>
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Este é o modelo GENÉRICO. Para vir com uma coluna por dia do evento, baixe pelo botão "Baixar modelo" da equipe, no sistema.</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Uma pessoa por linha, na aba "Equipe".</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Nome, CPF, Telefone (com DDD) e Cidade: obrigatórios. Cargo e Chave PIX: opcionais.</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Dias de trabalho (evento com escala por dia): as datas separadas por vírgula, ex.: 10/10, 11/10 — ou "todos".</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Quem ficar sem nenhum dia não é importado.</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>Não mude o nome das colunas e não deixe linha de exemplo: toda linha com nome é cadastrada.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A10"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>